<commit_message>
Split liste prix vente article.xlsx into 5 files of max 2000 rows with reference, designation, prix columns
Co-authored-by: dani679091817 <231127379+dani679091817@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/liste prix ventes articles part1.xlsx
+++ b/liste prix ventes articles part1.xlsx
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="C290" t="n">
-        <v>1200</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="291">
@@ -8494,7 +8494,7 @@
         </is>
       </c>
       <c r="C539" t="n">
-        <v>800</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="540">
@@ -10920,7 +10920,7 @@
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>CUILLIERE JETABLE LOT*50</t>
+          <t>CUILLERE JETABLE LOT*50</t>
         </is>
       </c>
       <c r="C701" t="n">
@@ -20929,7 +20929,7 @@
         </is>
       </c>
       <c r="C1368" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="1369">
@@ -22579,7 +22579,7 @@
         </is>
       </c>
       <c r="C1478" t="n">
-        <v>1450</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="1479">
@@ -22594,7 +22594,7 @@
         </is>
       </c>
       <c r="C1479" t="n">
-        <v>2700</v>
+        <v>3100</v>
       </c>
     </row>
     <row r="1480">

</xml_diff>